<commit_message>
Match NL IDs on sending country too; fix B36 org code
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Wo4ojnwbQsm1hctNz56575
</commit_message>
<xml_diff>
--- a/output/NL_291026_with_IDs.xlsx
+++ b/output/NL_291026_with_IDs.xlsx
@@ -2219,11 +2219,11 @@
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>7202</v>
+        <v>7204</v>
       </c>
       <c r="B36" s="7" t="inlineStr">
         <is>
-          <t>3PLDBSNL</t>
+          <t>3PLDBSBRNL</t>
         </is>
       </c>
       <c r="D36" s="7" t="inlineStr">

</xml_diff>